<commit_message>
paper run 2026-09-02 11:59
</commit_message>
<xml_diff>
--- a/reports/2026-09-02.xlsx
+++ b/reports/2026-09-02.xlsx
@@ -872,7 +872,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1025,13 +1025,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D15" t="n">
-        <v>99.75</v>
+        <v>52.98</v>
       </c>
       <c r="E15" t="n">
         <v>82.90000000000001</v>
@@ -1108,13 +1108,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D20" t="n">
-        <v>23.4</v>
+        <v>10.47</v>
       </c>
       <c r="E20" t="n">
         <v>2.45</v>
@@ -1123,50 +1123,62 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" t="n">
+        <v>-33.84</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>11</v>
-      </c>
-      <c r="C22" t="n">
-        <v>11</v>
-      </c>
-      <c r="D22" t="n">
-        <v>281.98</v>
-      </c>
-      <c r="E22" t="n">
-        <v>195.13</v>
+          <t>По цене входа</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>13</v>
+      </c>
+      <c r="C23" t="n">
+        <v>11</v>
+      </c>
+      <c r="D23" t="n">
+        <v>214.3</v>
+      </c>
+      <c r="E23" t="n">
+        <v>195.13</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>MAX_PER_WINDOW</t>
+          <t>0.60–0.62</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D24" t="n">
-        <v>49.05</v>
+        <v>20.91</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -1175,249 +1187,256 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>9</v>
-      </c>
-      <c r="C25" t="n">
-        <v>9</v>
-      </c>
-      <c r="D25" t="n">
-        <v>232.93</v>
-      </c>
-      <c r="E25" t="n">
-        <v>195.13</v>
+          <t>По риск-гейтам</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>MAX_PER_WINDOW</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>2</v>
+      </c>
+      <c r="C26" t="n">
+        <v>2</v>
+      </c>
+      <c r="D26" t="n">
+        <v>49.05</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>REALIZED (реальные сделки)</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>3</v>
+      </c>
+      <c r="C27" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" t="n">
+        <v>-46.77</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>9</v>
+      </c>
+      <c r="C28" t="n">
+        <v>9</v>
+      </c>
+      <c r="D28" t="n">
+        <v>232.93</v>
+      </c>
+      <c r="E28" t="n">
+        <v>195.13</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>BTC</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>8</v>
-      </c>
-      <c r="C30" t="n">
-        <v>8</v>
-      </c>
-      <c r="D30" t="n">
-        <v>192.68</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>SOL</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>1</v>
-      </c>
-      <c r="C31" t="n">
-        <v>1</v>
-      </c>
-      <c r="D31" t="n">
-        <v>2.45</v>
+          <t>REALIZED (реальные сделки)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>По активам</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>8</v>
+      </c>
+      <c r="C33" t="n">
+        <v>8</v>
+      </c>
+      <c r="D33" t="n">
+        <v>192.68</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>15m</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C34" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D34" t="n">
-        <v>82.90000000000001</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>5m</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>5</v>
-      </c>
-      <c r="C35" t="n">
-        <v>5</v>
-      </c>
-      <c r="D35" t="n">
-        <v>112.23</v>
+        <v>2.45</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>4</v>
+      </c>
+      <c r="C37" t="n">
+        <v>4</v>
+      </c>
+      <c r="D37" t="n">
+        <v>82.90000000000001</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>5m</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C38" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D38" t="n">
-        <v>31.23</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>5</v>
-      </c>
-      <c r="C39" t="n">
-        <v>5</v>
-      </c>
-      <c r="D39" t="n">
-        <v>132.88</v>
+        <v>112.23</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
-        <v>1</v>
-      </c>
-      <c r="C40" t="n">
-        <v>1</v>
-      </c>
-      <c r="D40" t="n">
-        <v>31.02</v>
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>3</v>
+      </c>
+      <c r="C41" t="n">
+        <v>3</v>
+      </c>
+      <c r="D41" t="n">
+        <v>31.23</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>5</v>
+      </c>
+      <c r="C42" t="n">
+        <v>5</v>
+      </c>
+      <c r="D42" t="n">
+        <v>132.88</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
+          <t>03</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="C43" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D43" t="n">
-        <v>195.13</v>
+        <v>31.02</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>По силе движения</t>
+          <t>По цене входа</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1439,118 +1458,156 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>0.10–0.12%</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C46" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D46" t="n">
-        <v>103.34</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>0.12–0.15%</t>
-        </is>
-      </c>
-      <c r="B47" t="n">
-        <v>2</v>
-      </c>
-      <c r="C47" t="n">
-        <v>2</v>
-      </c>
-      <c r="D47" t="n">
-        <v>59.32</v>
+        <v>195.13</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>0.15–0.20%</t>
-        </is>
-      </c>
-      <c r="B48" t="n">
-        <v>1</v>
-      </c>
-      <c r="C48" t="n">
-        <v>1</v>
-      </c>
-      <c r="D48" t="n">
-        <v>24.64</v>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>0.20%+</t>
+          <t>0.10–0.12%</t>
         </is>
       </c>
       <c r="B49" t="n">
+        <v>4</v>
+      </c>
+      <c r="C49" t="n">
+        <v>4</v>
+      </c>
+      <c r="D49" t="n">
+        <v>103.34</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
         <v>2</v>
       </c>
-      <c r="C49" t="n">
+      <c r="C50" t="n">
         <v>2</v>
       </c>
-      <c r="D49" t="n">
-        <v>7.83</v>
+      <c r="D50" t="n">
+        <v>59.32</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>0.15–0.20%</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" t="n">
+        <v>24.64</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
+          <t>0.20%+</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>2</v>
+      </c>
+      <c r="C52" t="n">
+        <v>2</v>
+      </c>
+      <c r="D52" t="n">
+        <v>7.83</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="B52" t="n">
+      <c r="B55" t="n">
         <v>1</v>
       </c>
-      <c r="C52" t="n">
+      <c r="C55" t="n">
         <v>1</v>
       </c>
-      <c r="D52" t="n">
+      <c r="D55" t="n">
         <v>5.38</v>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
+    <row r="56">
+      <c r="A56" t="inlineStr">
         <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="B53" t="n">
+      <c r="B56" t="n">
         <v>8</v>
       </c>
-      <c r="C53" t="n">
+      <c r="C56" t="n">
         <v>8</v>
       </c>
-      <c r="D53" t="n">
+      <c r="D56" t="n">
         <v>189.75</v>
       </c>
     </row>

</xml_diff>

<commit_message>
paper run 2026-09-02 17:55
</commit_message>
<xml_diff>
--- a/reports/2026-09-02.xlsx
+++ b/reports/2026-09-02.xlsx
@@ -872,7 +872,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1025,13 +1025,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C15" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D15" t="n">
-        <v>52.98</v>
+        <v>139.46</v>
       </c>
       <c r="E15" t="n">
         <v>82.90000000000001</v>
@@ -1044,13 +1044,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C16" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D16" t="n">
-        <v>182.23</v>
+        <v>232.15</v>
       </c>
       <c r="E16" t="n">
         <v>112.23</v>
@@ -1089,13 +1089,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D19" t="n">
-        <v>25.65</v>
+        <v>59.49</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
@@ -1108,13 +1108,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C20" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D20" t="n">
-        <v>10.47</v>
+        <v>62.99</v>
       </c>
       <c r="E20" t="n">
         <v>2.45</v>
@@ -1127,13 +1127,13 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D21" t="n">
-        <v>-33.84</v>
+        <v>16.2</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
@@ -1153,13 +1153,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C23" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D23" t="n">
-        <v>214.3</v>
+        <v>313.22</v>
       </c>
       <c r="E23" t="n">
         <v>195.13</v>
@@ -1168,7 +1168,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0.60–0.62</t>
+          <t>0.55–0.60</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1178,7 +1178,7 @@
         <v>1</v>
       </c>
       <c r="D24" t="n">
-        <v>20.91</v>
+        <v>18.8</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -1187,43 +1187,43 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>2</v>
+      </c>
+      <c r="C25" t="n">
+        <v>2</v>
+      </c>
+      <c r="D25" t="n">
+        <v>39.59</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>MAX_PER_WINDOW</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>2</v>
-      </c>
-      <c r="C26" t="n">
-        <v>2</v>
-      </c>
-      <c r="D26" t="n">
-        <v>49.05</v>
-      </c>
-      <c r="E26" t="n">
-        <v>0</v>
+          <t>По риск-гейтам</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>NO_LIQUIDITY</t>
+          <t>MAX_PER_WINDOW</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D27" t="n">
-        <v>-46.77</v>
+        <v>49.05</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
@@ -1232,382 +1232,401 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>8</v>
+      </c>
+      <c r="C28" t="n">
+        <v>6</v>
+      </c>
+      <c r="D28" t="n">
+        <v>89.63</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="B28" t="n">
+      <c r="B29" t="n">
         <v>9</v>
       </c>
-      <c r="C28" t="n">
+      <c r="C29" t="n">
         <v>9</v>
       </c>
-      <c r="D28" t="n">
+      <c r="D29" t="n">
         <v>232.93</v>
       </c>
-      <c r="E28" t="n">
+      <c r="E29" t="n">
         <v>195.13</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
+    <row r="31">
+      <c r="A31" t="inlineStr">
         <is>
           <t>REALIZED (реальные сделки)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>BTC</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>8</v>
-      </c>
-      <c r="C33" t="n">
-        <v>8</v>
-      </c>
-      <c r="D33" t="n">
-        <v>192.68</v>
+          <t>По активам</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>8</v>
+      </c>
+      <c r="C34" t="n">
+        <v>8</v>
+      </c>
+      <c r="D34" t="n">
+        <v>192.68</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>SOL</t>
         </is>
       </c>
-      <c r="B34" t="n">
+      <c r="B35" t="n">
         <v>1</v>
       </c>
-      <c r="C34" t="n">
+      <c r="C35" t="n">
         <v>1</v>
       </c>
-      <c r="D34" t="n">
+      <c r="D35" t="n">
         <v>2.45</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>15m</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>4</v>
-      </c>
-      <c r="C37" t="n">
-        <v>4</v>
-      </c>
-      <c r="D37" t="n">
-        <v>82.90000000000001</v>
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>4</v>
+      </c>
+      <c r="C38" t="n">
+        <v>4</v>
+      </c>
+      <c r="D38" t="n">
+        <v>82.90000000000001</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>5m</t>
         </is>
       </c>
-      <c r="B38" t="n">
+      <c r="B39" t="n">
         <v>5</v>
       </c>
-      <c r="C38" t="n">
+      <c r="C39" t="n">
         <v>5</v>
       </c>
-      <c r="D38" t="n">
+      <c r="D39" t="n">
         <v>112.23</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>3</v>
-      </c>
-      <c r="C41" t="n">
-        <v>3</v>
-      </c>
-      <c r="D41" t="n">
-        <v>31.23</v>
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>01</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C42" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D42" t="n">
-        <v>132.88</v>
+        <v>31.23</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>5</v>
+      </c>
+      <c r="C43" t="n">
+        <v>5</v>
+      </c>
+      <c r="D43" t="n">
+        <v>132.88</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
           <t>03</t>
         </is>
       </c>
-      <c r="B43" t="n">
+      <c r="B44" t="n">
         <v>1</v>
       </c>
-      <c r="C43" t="n">
+      <c r="C44" t="n">
         <v>1</v>
       </c>
-      <c r="D43" t="n">
+      <c r="D44" t="n">
         <v>31.02</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
           <t>0.50–0.55</t>
         </is>
       </c>
-      <c r="B46" t="n">
+      <c r="B47" t="n">
         <v>9</v>
       </c>
-      <c r="C46" t="n">
+      <c r="C47" t="n">
         <v>9</v>
       </c>
-      <c r="D46" t="n">
+      <c r="D47" t="n">
         <v>195.13</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>0.10–0.12%</t>
-        </is>
-      </c>
-      <c r="B49" t="n">
-        <v>4</v>
-      </c>
-      <c r="C49" t="n">
-        <v>4</v>
-      </c>
-      <c r="D49" t="n">
-        <v>103.34</v>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>0.12–0.15%</t>
+          <t>0.10–0.12%</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C50" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D50" t="n">
-        <v>59.32</v>
+        <v>103.34</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>0.15–0.20%</t>
+          <t>0.12–0.15%</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D51" t="n">
-        <v>24.64</v>
+        <v>59.32</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
+          <t>0.15–0.20%</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" t="n">
+        <v>24.64</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
           <t>0.20%+</t>
         </is>
       </c>
-      <c r="B52" t="n">
+      <c r="B53" t="n">
         <v>2</v>
       </c>
-      <c r="C52" t="n">
+      <c r="C53" t="n">
         <v>2</v>
       </c>
-      <c r="D52" t="n">
+      <c r="D53" t="n">
         <v>7.83</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>DOWN</t>
-        </is>
-      </c>
-      <c r="B55" t="n">
-        <v>1</v>
-      </c>
-      <c r="C55" t="n">
-        <v>1</v>
-      </c>
-      <c r="D55" t="n">
-        <v>5.38</v>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>1</v>
+      </c>
+      <c r="C56" t="n">
+        <v>1</v>
+      </c>
+      <c r="D56" t="n">
+        <v>5.38</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
           <t>UP</t>
         </is>
       </c>
-      <c r="B56" t="n">
+      <c r="B57" t="n">
         <v>8</v>
       </c>
-      <c r="C56" t="n">
+      <c r="C57" t="n">
         <v>8</v>
       </c>
-      <c r="D56" t="n">
+      <c r="D57" t="n">
         <v>189.75</v>
       </c>
     </row>

</xml_diff>

<commit_message>
paper run 2026-09-02 23:54
</commit_message>
<xml_diff>
--- a/reports/2026-09-02.xlsx
+++ b/reports/2026-09-02.xlsx
@@ -1025,13 +1025,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C15" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D15" t="n">
-        <v>139.46</v>
+        <v>173.3</v>
       </c>
       <c r="E15" t="n">
         <v>82.90000000000001</v>
@@ -1108,13 +1108,13 @@
         </is>
       </c>
       <c r="B20" t="n">
+        <v>6</v>
+      </c>
+      <c r="C20" t="n">
         <v>5</v>
       </c>
-      <c r="C20" t="n">
-        <v>4</v>
-      </c>
       <c r="D20" t="n">
-        <v>62.99</v>
+        <v>96.83</v>
       </c>
       <c r="E20" t="n">
         <v>2.45</v>
@@ -1153,13 +1153,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C23" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D23" t="n">
-        <v>313.22</v>
+        <v>347.06</v>
       </c>
       <c r="E23" t="n">
         <v>195.13</v>
@@ -1236,13 +1236,13 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C28" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D28" t="n">
-        <v>89.63</v>
+        <v>123.47</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>

</xml_diff>